<commit_message>
feat: add overview generator, macOS automation setup, and test data with overviews
</commit_message>
<xml_diff>
--- a/test_data/Details_April_2026.xlsx
+++ b/test_data/Details_April_2026.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Details April 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="April 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Details April 2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,8 +39,17 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +68,16 @@
         <bgColor rgb="00EBF3FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -82,6 +102,11 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,6 +472,521 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:M12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Resource Name</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>POD Name</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Work Package Code</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Week 1</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Week 3</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>Week 4</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>Total Hours</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>Fee</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>Group PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Edmund Blackadder</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Cobra POD</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.11</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="n">
+        <v>185</v>
+      </c>
+      <c r="F3" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" s="10" t="n"/>
+      <c r="H3" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="J3" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="K3" s="10">
+        <f>SUM(F3:J3)</f>
+        <v/>
+      </c>
+      <c r="L3" s="10">
+        <f>K3*E3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>S. Baldrick</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Cobra POD</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.11</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="F4" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="H4" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="I4" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="J4" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="K4" s="10">
+        <f>SUM(F4:J4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="10">
+        <f>K4*E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>George St. Barleigh</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Cobra POD</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.11</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>130</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="K5" s="10">
+        <f>SUM(F5:J5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="10">
+        <f>K5*E5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Nurse Darling</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Viper POD</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.22</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>140</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="K6" s="10">
+        <f>SUM(F6:J6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="10">
+        <f>K6*E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Gen. Melchett</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Viper POD</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.22</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="K7" s="10">
+        <f>SUM(F7:J7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="10">
+        <f>K7*E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Capt. Kevin Darling</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Viper POD</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.22</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="K8" s="10">
+        <f>SUM(F8:J8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="10">
+        <f>K8*E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Bobbie Parkhurst</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Python POD</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.33</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>125</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="J9" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="K9" s="10">
+        <f>SUM(F9:J9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="10">
+        <f>K9*E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Lord Percy Percy</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Python POD</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.33</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>145</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="K10" s="10">
+        <f>SUM(F10:J10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="10">
+        <f>K10*E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Mrs. Miggins</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Cobra POD</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>GBL0007741.2.11</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>115</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="K11" s="10">
+        <f>SUM(F11:J11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="10">
+        <f>K11*E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="11">
+        <f>SUM(F3:F11)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11">
+        <f>SUM(G3:G11)</f>
+        <v/>
+      </c>
+      <c r="H12" s="11">
+        <f>SUM(H3:H11)</f>
+        <v/>
+      </c>
+      <c r="I12" s="11">
+        <f>SUM(I3:I11)</f>
+        <v/>
+      </c>
+      <c r="J12" s="11">
+        <f>SUM(J3:J11)</f>
+        <v/>
+      </c>
+      <c r="K12" s="11">
+        <f>SUM(K3:K11)</f>
+        <v/>
+      </c>
+      <c r="L12" s="11">
+        <f>SUM(L3:L11)</f>
+        <v/>
+      </c>
+      <c r="M12" s="12" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>